<commit_message>
Update news database from Excel
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trece\Documents\Code\unked\mi-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CC7FB5-BE62-4E5C-886F-078F2D57D9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D9C63B-6BD3-4D14-BE83-14A56DE141DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{15C9D418-315A-4B88-91DE-BBEFAE06072D}"/>
+    <workbookView xWindow="7305" yWindow="0" windowWidth="21600" windowHeight="11835" xr2:uid="{15C9D418-315A-4B88-91DE-BBEFAE06072D}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="2" r:id="rId1"/>
@@ -28030,7 +28030,7 @@
       </c>
       <c r="G278" s="1"/>
       <c r="H278" s="1">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="I278" s="1" t="s">
         <v>1459</v>

</xml_diff>

<commit_message>
Refactor: Navigation tactile effects, Article styles and BBDD Update
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5725835-0323-4794-B0C7-B836627682E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6594E5E4-F67C-4ACA-9767-CE6F4C28FAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="2" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="1509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="1518">
   <si>
     <t>id</t>
   </si>
@@ -18430,6 +18430,77 @@
   </si>
   <si>
     <t>https://i.postimg.cc/htGbkgSZ/497.png</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXKMHZmk-8g/</t>
+  </si>
+  <si>
+    <t>Cuando se habla de fútbol, no todo está inventando. Aquí vemos a Jan Virgili del Mallorca marcando con los dos pies a la vez.</t>
+  </si>
+  <si>
+    <t>El RCD Mallorca se enfrentó al Rayo Vallecano este domingo pasado y lo goleó 3-0 con dos goles del pirata del gol, Vedat Muriqi, y otro gol de Jan Virgili.</t>
+  </si>
+  <si>
+    <t>Este último gol se dio en el minuto 65 tras un centro al área de Pablo Torre, al que Virgili respondió pateando con los dos pies a la vez.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Gol de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jan Virgili</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> con los </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dos pies</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a la vez</t>
+    </r>
+  </si>
+  <si>
+    <t>mallorca, laliga, jan virgili</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/zDTMMbWW/494.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/Sx5JnNdf/462.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/DwD8Sy6c/464.png</t>
   </si>
 </sst>
 </file>
@@ -18502,7 +18573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -18510,6 +18581,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18844,7 +18916,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S278"/>
+  <dimension ref="A1:S279"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -19959,7 +20031,7 @@
         <v>46047</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>168</v>
+        <v>73</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>169</v>
@@ -27569,6 +27641,9 @@
       <c r="I264" s="1" t="s">
         <v>1389</v>
       </c>
+      <c r="J264" s="7" t="s">
+        <v>1516</v>
+      </c>
       <c r="K264" s="3" t="s">
         <v>1390</v>
       </c>
@@ -27605,6 +27680,9 @@
       <c r="I265" s="1" t="s">
         <v>1395</v>
       </c>
+      <c r="J265" s="6" t="s">
+        <v>1517</v>
+      </c>
       <c r="K265" s="3" t="s">
         <v>1396</v>
       </c>
@@ -28035,7 +28113,7 @@
       </c>
       <c r="G276" s="1"/>
       <c r="H276" s="1">
-        <v>922000</v>
+        <v>1000000</v>
       </c>
       <c r="I276" s="1" t="s">
         <v>1477</v>
@@ -28074,7 +28152,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>4000000</v>
+        <v>5000000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28096,44 +28174,83 @@
       <c r="A278">
         <v>277</v>
       </c>
-      <c r="B278" s="6">
-        <v>497</v>
+      <c r="B278" s="1">
+        <v>494</v>
       </c>
       <c r="C278" s="2">
-        <v>46128</v>
+        <v>46127</v>
       </c>
       <c r="D278" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E278" s="6" t="s">
+        <v>1514</v>
+      </c>
+      <c r="F278" s="6" t="s">
+        <v>1513</v>
+      </c>
+      <c r="G278" s="6"/>
+      <c r="H278" s="1">
+        <v>250000</v>
+      </c>
+      <c r="I278" s="6" t="s">
+        <v>1509</v>
+      </c>
+      <c r="J278" s="6" t="s">
+        <v>1515</v>
+      </c>
+      <c r="K278" s="3" t="s">
+        <v>1510</v>
+      </c>
+      <c r="L278" s="3" t="s">
+        <v>1511</v>
+      </c>
+      <c r="M278" s="3" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="279" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A279">
+        <v>278</v>
+      </c>
+      <c r="B279" s="6">
+        <v>497</v>
+      </c>
+      <c r="C279" s="2">
+        <v>46128</v>
+      </c>
+      <c r="D279" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E279" s="6" t="s">
         <v>1504</v>
       </c>
-      <c r="F278" s="6" t="s">
+      <c r="F279" s="6" t="s">
         <v>1503</v>
       </c>
-      <c r="G278" s="6"/>
-      <c r="H278" s="6">
-        <v>369000</v>
-      </c>
-      <c r="I278" s="6" t="s">
+      <c r="G279" s="6"/>
+      <c r="H279" s="6">
+        <v>950000</v>
+      </c>
+      <c r="I279" s="6" t="s">
         <v>1502</v>
       </c>
-      <c r="J278" s="6" t="s">
+      <c r="J279" s="6" t="s">
         <v>1508</v>
       </c>
-      <c r="K278" s="3" t="s">
+      <c r="K279" s="3" t="s">
         <v>1505</v>
       </c>
-      <c r="L278" s="3" t="s">
+      <c r="L279" s="3" t="s">
         <v>1506</v>
       </c>
-      <c r="M278" s="3" t="s">
+      <c r="M279" s="3" t="s">
         <v>1507</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Actualización de base de datos desde Excel
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6594E5E4-F67C-4ACA-9767-CE6F4C28FAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB31C76-9142-4C8A-94E7-E19191EF0CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="1518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="1538">
   <si>
     <t>id</t>
   </si>
@@ -18501,6 +18501,186 @@
   </si>
   <si>
     <t>https://i.postimg.cc/DwD8Sy6c/464.png</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXPpIl8E3Bn/</t>
+  </si>
+  <si>
+    <t>Esto ha ocurrido en la fase de grupos de la CONMEBOL Sudamericana.</t>
+  </si>
+  <si>
+    <t>EL Red Bull Bragantino de Brasil se ha enfrentado al Blooming de Bolivia cuando el argentino Diago Giménez ha cometido dos entradas dignas de carnicero a dos jugadores del Bragantino.</t>
+  </si>
+  <si>
+    <t>Insólito que tras esas dos entradas, encima se quejara al árbitro por su decisión de sacar dos tarjetas amarillas seguidas con su consiguiente expulsión.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2 tarjetas amarillas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en la misma jugada, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tarjeta roja</t>
+    </r>
+  </si>
+  <si>
+    <t>conmebol, brasil, argentina, bolivia</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXRGrC5E2p3/</t>
+  </si>
+  <si>
+    <t>¿Quién tiene más mala suerte, una víctima de la isla de Jeffrey Epstein o Pedro Buenpito?</t>
+  </si>
+  <si>
+    <t>En el último partido del Real Murcia en Primera RFEF, el delantero Pedro Benito tuvo la mala suerte de que una irregularidad en el césped le despejara un chute que iba directo a la red.</t>
+  </si>
+  <si>
+    <t>Para más inri, el partido acabó 2-3 a favor del Antequera, así que este gol hubiese cambiado el resultado de derrota a empate.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>césped</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> despeja un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gol</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> que estaba casi </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>asegurado</t>
+    </r>
+  </si>
+  <si>
+    <t>primera rfef, real murcia, pedro benito</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXR-2q1E8Ox/</t>
+  </si>
+  <si>
+    <t>Así actúa un buen capitán. Como hizo Natxo Insa, el futbolista que pasó por equipos como el RC Celta, Valencia CF, Real Zaragoza o Levante UD.</t>
+  </si>
+  <si>
+    <t>Jugó ayer con su equipo, el Johor DT, en la primera división de Malasia, y pudimos ver su frustración cuando su compañero Jairo se encontraba en el suelo y pese a que pedían atención médica nadie del staff médico reaccionaba.</t>
+  </si>
+  <si>
+    <t>Como buen capitán, hizo todo lo posible para darle solución. Fue a quitarle el banderín al árbitro, y pegó un sprint para llegar donde los médicos y pateó al camillero para que despertara y fueran a atender a su compañero.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Lo que haga falta para que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>atiendan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a su </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>compañero</t>
+    </r>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/Y07LYNPv/502.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/7h4J01RC/503.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/6qK4nVPy/505.png</t>
   </si>
 </sst>
 </file>
@@ -18573,7 +18753,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -18581,7 +18761,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18916,7 +19095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S279"/>
+  <dimension ref="A1:S282"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -27641,7 +27820,7 @@
       <c r="I264" s="1" t="s">
         <v>1389</v>
       </c>
-      <c r="J264" s="7" t="s">
+      <c r="J264" s="6" t="s">
         <v>1516</v>
       </c>
       <c r="K264" s="3" t="s">
@@ -28246,6 +28425,119 @@
       </c>
       <c r="M279" s="3" t="s">
         <v>1507</v>
+      </c>
+    </row>
+    <row r="280" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A280">
+        <v>279</v>
+      </c>
+      <c r="B280" s="6">
+        <v>502</v>
+      </c>
+      <c r="C280" s="2">
+        <v>46129</v>
+      </c>
+      <c r="D280" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E280" s="6" t="s">
+        <v>1523</v>
+      </c>
+      <c r="F280" s="6" t="s">
+        <v>1522</v>
+      </c>
+      <c r="G280" s="6"/>
+      <c r="H280" s="6">
+        <v>101000</v>
+      </c>
+      <c r="I280" s="6" t="s">
+        <v>1518</v>
+      </c>
+      <c r="J280" s="6" t="s">
+        <v>1535</v>
+      </c>
+      <c r="K280" s="3" t="s">
+        <v>1519</v>
+      </c>
+      <c r="L280" s="3" t="s">
+        <v>1520</v>
+      </c>
+      <c r="M280" s="3" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="281" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" s="6">
+        <v>503</v>
+      </c>
+      <c r="C281" s="2">
+        <v>46129</v>
+      </c>
+      <c r="D281" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E281" s="6" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F281" s="6" t="s">
+        <v>1528</v>
+      </c>
+      <c r="G281" s="6"/>
+      <c r="H281" s="6">
+        <v>100000</v>
+      </c>
+      <c r="I281" s="6" t="s">
+        <v>1524</v>
+      </c>
+      <c r="J281" s="6" t="s">
+        <v>1536</v>
+      </c>
+      <c r="K281" s="3" t="s">
+        <v>1525</v>
+      </c>
+      <c r="L281" s="3" t="s">
+        <v>1526</v>
+      </c>
+      <c r="M281" s="3" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="282" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A282">
+        <v>281</v>
+      </c>
+      <c r="B282" s="6">
+        <v>505</v>
+      </c>
+      <c r="C282" s="2">
+        <v>46130</v>
+      </c>
+      <c r="D282" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F282" s="6" t="s">
+        <v>1534</v>
+      </c>
+      <c r="H282" s="6">
+        <v>1500000</v>
+      </c>
+      <c r="I282" s="6" t="s">
+        <v>1530</v>
+      </c>
+      <c r="J282" s="6" t="s">
+        <v>1537</v>
+      </c>
+      <c r="K282" s="3" t="s">
+        <v>1531</v>
+      </c>
+      <c r="L282" s="3" t="s">
+        <v>1532</v>
+      </c>
+      <c r="M282" s="3" t="s">
+        <v>1533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización de base de datos desde Excel (re-ejecución)
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB31C76-9142-4C8A-94E7-E19191EF0CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463F0708-2283-4EAC-89BF-AD9E188ABDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28292,7 +28292,7 @@
       </c>
       <c r="G276" s="1"/>
       <c r="H276" s="1">
-        <v>1000000</v>
+        <v>1100000</v>
       </c>
       <c r="I276" s="1" t="s">
         <v>1477</v>
@@ -28331,7 +28331,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>5000000</v>
+        <v>5500000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28370,7 +28370,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>250000</v>
+        <v>402000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28409,7 +28409,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>950000</v>
+        <v>973000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>

</xml_diff>

<commit_message>
Actualización de base de datos desde Excel (tercera ejecución)
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463F0708-2283-4EAC-89BF-AD9E188ABDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C32FB9-F32C-41D5-BBE9-0ED1ECD3E9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27005,7 +27005,7 @@
       </c>
       <c r="G242" s="1"/>
       <c r="H242" s="1">
-        <v>588000</v>
+        <v>589000</v>
       </c>
       <c r="I242" s="1" t="s">
         <v>1249</v>
@@ -27445,7 +27445,7 @@
       </c>
       <c r="G254" s="1"/>
       <c r="H254" s="1">
-        <v>254000</v>
+        <v>255000</v>
       </c>
       <c r="I254" s="1" t="s">
         <v>1325</v>
@@ -27519,7 +27519,7 @@
         <v>1336</v>
       </c>
       <c r="H256" s="1">
-        <v>742000</v>
+        <v>743000</v>
       </c>
       <c r="I256" s="1" t="s">
         <v>1337</v>
@@ -27740,7 +27740,7 @@
       </c>
       <c r="G262" s="1"/>
       <c r="H262" s="1">
-        <v>500000</v>
+        <v>501000</v>
       </c>
       <c r="I262" s="1" t="s">
         <v>1376</v>
@@ -27815,7 +27815,7 @@
       </c>
       <c r="G264" s="1"/>
       <c r="H264" s="1">
-        <v>134000</v>
+        <v>135000</v>
       </c>
       <c r="I264" s="1" t="s">
         <v>1389</v>
@@ -27890,7 +27890,7 @@
       </c>
       <c r="G266" s="1"/>
       <c r="H266" s="1">
-        <v>182000</v>
+        <v>183000</v>
       </c>
       <c r="I266" s="1" t="s">
         <v>1400</v>
@@ -27974,7 +27974,7 @@
       </c>
       <c r="G268" s="1"/>
       <c r="H268" s="1">
-        <v>100000</v>
+        <v>101000</v>
       </c>
       <c r="I268" s="1" t="s">
         <v>1417</v>
@@ -28051,7 +28051,7 @@
         <v>1431</v>
       </c>
       <c r="H270" s="1">
-        <v>59000</v>
+        <v>60000</v>
       </c>
       <c r="I270" s="1" t="s">
         <v>1432</v>
@@ -28129,7 +28129,7 @@
       </c>
       <c r="G272" s="1"/>
       <c r="H272" s="1">
-        <v>731000</v>
+        <v>733000</v>
       </c>
       <c r="I272" s="1" t="s">
         <v>1446</v>
@@ -28170,7 +28170,7 @@
         <v>1453</v>
       </c>
       <c r="H273" s="1">
-        <v>331000</v>
+        <v>332000</v>
       </c>
       <c r="I273" s="1" t="s">
         <v>1454</v>
@@ -28209,7 +28209,7 @@
       </c>
       <c r="G274" s="1"/>
       <c r="H274" s="1">
-        <v>204000</v>
+        <v>205000</v>
       </c>
       <c r="I274" s="1" t="s">
         <v>1461</v>
@@ -28250,7 +28250,7 @@
         <v>1468</v>
       </c>
       <c r="H275" s="1">
-        <v>788000</v>
+        <v>789000</v>
       </c>
       <c r="I275" s="1" t="s">
         <v>1469</v>

</xml_diff>

<commit_message>
Actualización periódica de base de datos desde Excel
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C32FB9-F32C-41D5-BBE9-0ED1ECD3E9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD126E1-EDFD-4559-AD82-907E91D3A0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28370,7 +28370,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>402000</v>
+        <v>412000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28448,7 +28448,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>101000</v>
+        <v>102000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1518</v>
@@ -28522,7 +28522,7 @@
         <v>1534</v>
       </c>
       <c r="H282" s="6">
-        <v>1500000</v>
+        <v>1600000</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>1530</v>

</xml_diff>

<commit_message>
Actualización manual de base de datos desde Excel
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD126E1-EDFD-4559-AD82-907E91D3A0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67E34C-0F1E-42B9-B9AB-EC81A75835E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="2" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="1538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1791" uniqueCount="1553">
   <si>
     <t>id</t>
   </si>
@@ -18681,6 +18681,157 @@
   </si>
   <si>
     <t>https://i.postimg.cc/6qK4nVPy/505.png</t>
+  </si>
+  <si>
+    <t>copa del rey, atleti, cholo simeone, real sociedad</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXTxWhmk9Ok/</t>
+  </si>
+  <si>
+    <t>Esa es la Cholo Mentality.</t>
+  </si>
+  <si>
+    <t>Anoche se jugó la final de la Copa del Rey entre el Atlético de Madrid y la Real Sociedad, encuentro que terminó 2-2 y se decidió en penaltis, donde la Real se impuso y acabó alzando la copa.</t>
+  </si>
+  <si>
+    <t>Se trata de una final que el Cholo Simeone ha estado persiguiendo durante los últimos 13 años, y el primer tanto del equipo rival llegó a tan solo 14 segundos del pitido inicial. Pechofriada histórica del argentino.</t>
+  </si>
+  <si>
+    <r>
+      <t>13 años</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> persiguiendo una </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>final</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>copa</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para que te marquen a los </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>14 segundos</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXT6fJ1E5L5/</t>
+  </si>
+  <si>
+    <t>Cada jugador tiene sus tácticas para rendir más en el terreno de juego.</t>
+  </si>
+  <si>
+    <t>En la final de la Copa del Rey entre el Atlético de Madrid y la Real Sociedad, pudimos ver a Oyarzabal aplicando métodos que le han funcionado de forma regular a Bellingham, pero al parecer a él le sirvió para activar el modo Terreneitor y llevarse la copa.</t>
+  </si>
+  <si>
+    <t>Darío Eme Hache, que se encontraba narrando la retransmisión del partido junto a Ibai Llanos en su canal, se percató del suceso y comentó: "No hombre no, para rendir cubatas no, es mucho mejor darle a la línea de cal".</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Oyarzabal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> potando el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ron negrita</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para reactivarse</t>
+    </r>
+  </si>
+  <si>
+    <t>Cositas de Bellingham</t>
+  </si>
+  <si>
+    <t>copa del rey, atleti, real sociedad, oyarzabal</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/MKsp1sW6/506.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/MKsp1sWZ/507.png</t>
   </si>
 </sst>
 </file>
@@ -19095,7 +19246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S282"/>
+  <dimension ref="A1:S284"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -28331,7 +28482,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>5500000</v>
+        <v>5600000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28370,7 +28521,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>412000</v>
+        <v>440000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28409,7 +28560,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>973000</v>
+        <v>975000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28448,7 +28599,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>102000</v>
+        <v>107000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1518</v>
@@ -28487,7 +28638,7 @@
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>100000</v>
+        <v>109000</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>1524</v>
@@ -28521,8 +28672,9 @@
       <c r="F282" s="6" t="s">
         <v>1534</v>
       </c>
+      <c r="G282" s="6"/>
       <c r="H282" s="6">
-        <v>1600000</v>
+        <v>2200000</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>1530</v>
@@ -28538,6 +28690,86 @@
       </c>
       <c r="M282" s="3" t="s">
         <v>1533</v>
+      </c>
+    </row>
+    <row r="283" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A283">
+        <v>282</v>
+      </c>
+      <c r="B283" s="6">
+        <v>506</v>
+      </c>
+      <c r="C283" s="2">
+        <v>46131</v>
+      </c>
+      <c r="D283" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E283" s="6" t="s">
+        <v>1538</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>1543</v>
+      </c>
+      <c r="G283" s="6"/>
+      <c r="H283" s="6">
+        <v>85000</v>
+      </c>
+      <c r="I283" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="J283" s="6" t="s">
+        <v>1551</v>
+      </c>
+      <c r="K283" s="3" t="s">
+        <v>1540</v>
+      </c>
+      <c r="L283" s="3" t="s">
+        <v>1541</v>
+      </c>
+      <c r="M283" s="3" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="284" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" s="6">
+        <v>507</v>
+      </c>
+      <c r="C284" s="2">
+        <v>46131</v>
+      </c>
+      <c r="D284" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E284" s="6" t="s">
+        <v>1550</v>
+      </c>
+      <c r="F284" s="6" t="s">
+        <v>1548</v>
+      </c>
+      <c r="G284" s="6" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H284" s="6">
+        <v>100000</v>
+      </c>
+      <c r="I284" s="6" t="s">
+        <v>1544</v>
+      </c>
+      <c r="J284" s="6" t="s">
+        <v>1552</v>
+      </c>
+      <c r="K284" s="3" t="s">
+        <v>1545</v>
+      </c>
+      <c r="L284" s="3" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M284" s="3" t="s">
+        <v>1547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update news database and refine Instagram logo styling
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB127B43-07EB-4FE7-A78F-4630A47C2F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626815E1-9F39-48B5-900E-9595FC89513E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="2" r:id="rId1"/>
@@ -28521,7 +28521,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>447000</v>
+        <v>456000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28560,7 +28560,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>975000</v>
+        <v>976000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28599,7 +28599,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>108000</v>
+        <v>110000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1518</v>
@@ -28638,7 +28638,7 @@
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>111000</v>
+        <v>113000</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>1524</v>
@@ -28713,7 +28713,7 @@
       </c>
       <c r="G283" s="6"/>
       <c r="H283" s="6">
-        <v>100000</v>
+        <v>125000</v>
       </c>
       <c r="I283" s="6" t="s">
         <v>1539</v>
@@ -28754,7 +28754,7 @@
         <v>1549</v>
       </c>
       <c r="H284" s="6">
-        <v>115000</v>
+        <v>149000</v>
       </c>
       <c r="I284" s="6" t="s">
         <v>1544</v>

</xml_diff>

<commit_message>
Update database and increase Instagram logo size to w-14
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626815E1-9F39-48B5-900E-9595FC89513E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E92998-A571-4ACC-A89E-3217BE0042D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28482,7 +28482,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>5600000</v>
+        <v>5700000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28521,7 +28521,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>456000</v>
+        <v>498000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28560,7 +28560,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>976000</v>
+        <v>978000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28599,7 +28599,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>110000</v>
+        <v>114000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1518</v>
@@ -28638,7 +28638,7 @@
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>113000</v>
+        <v>121000</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>1524</v>
@@ -28713,7 +28713,7 @@
       </c>
       <c r="G283" s="6"/>
       <c r="H283" s="6">
-        <v>125000</v>
+        <v>215000</v>
       </c>
       <c r="I283" s="6" t="s">
         <v>1539</v>
@@ -28754,7 +28754,7 @@
         <v>1549</v>
       </c>
       <c r="H284" s="6">
-        <v>149000</v>
+        <v>271000</v>
       </c>
       <c r="I284" s="6" t="s">
         <v>1544</v>

</xml_diff>

<commit_message>
Update database and sync news
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F12C30-5160-4E8D-B0F1-2CC6C5F6FD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A2FFB4-913E-4F6E-92AB-F484577A4D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLA" sheetId="2" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="1560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="1566">
   <si>
     <t>id</t>
   </si>
@@ -18926,6 +18926,58 @@
   </si>
   <si>
     <t>https://i.postimg.cc/MKtJbB5Y/508.png</t>
+  </si>
+  <si>
+    <t>chiringuito, brad pitt, juanma rodríguez</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Para cuando te hablen de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>injusticias</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>fútbol</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXPXiLKDPtM/</t>
+  </si>
+  <si>
+    <t>Hablando sobre el partido de Bayern de Múnich - Real Madrid de Champions en el programa de radio El Primer Palo, el reconocido periodista Juanma Rodríguez tuvo que dar su opinión.</t>
+  </si>
+  <si>
+    <t>El también tertuliano de El Chiringuito de Jugones dio su opinión sobre el concepto de argumentar de justicia o injusticia en el fútbol extrapolándolo a una temática más cruda y real.</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/kgVpv5G5/501.png</t>
   </si>
 </sst>
 </file>
@@ -19340,7 +19392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S285"/>
+  <dimension ref="A1:S286"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -28576,7 +28628,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>6100000</v>
+        <v>7000000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28615,7 +28667,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>625000</v>
+        <v>917000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28654,7 +28706,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>982000</v>
+        <v>997000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28677,7 +28729,7 @@
         <v>279</v>
       </c>
       <c r="B280" s="6">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C280" s="2">
         <v>46129</v>
@@ -28686,29 +28738,26 @@
         <v>39</v>
       </c>
       <c r="E280" s="6" t="s">
-        <v>1523</v>
+        <v>1560</v>
       </c>
       <c r="F280" s="6" t="s">
-        <v>1522</v>
+        <v>1561</v>
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>128000</v>
+        <v>87000</v>
       </c>
       <c r="I280" s="6" t="s">
-        <v>1518</v>
+        <v>1562</v>
       </c>
       <c r="J280" s="6" t="s">
-        <v>1535</v>
+        <v>1565</v>
       </c>
       <c r="K280" s="3" t="s">
-        <v>1519</v>
+        <v>1563</v>
       </c>
       <c r="L280" s="3" t="s">
-        <v>1520</v>
-      </c>
-      <c r="M280" s="3" t="s">
-        <v>1521</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="281" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -28716,7 +28765,7 @@
         <v>280</v>
       </c>
       <c r="B281" s="6">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C281" s="2">
         <v>46129</v>
@@ -28725,29 +28774,29 @@
         <v>39</v>
       </c>
       <c r="E281" s="6" t="s">
-        <v>1529</v>
+        <v>1523</v>
       </c>
       <c r="F281" s="6" t="s">
-        <v>1528</v>
+        <v>1522</v>
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>136000</v>
+        <v>188000</v>
       </c>
       <c r="I281" s="6" t="s">
-        <v>1524</v>
+        <v>1518</v>
       </c>
       <c r="J281" s="6" t="s">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="K281" s="3" t="s">
-        <v>1525</v>
+        <v>1519</v>
       </c>
       <c r="L281" s="3" t="s">
-        <v>1526</v>
+        <v>1520</v>
       </c>
       <c r="M281" s="3" t="s">
-        <v>1527</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="282" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -28755,35 +28804,38 @@
         <v>281</v>
       </c>
       <c r="B282" s="6">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C282" s="2">
-        <v>46130</v>
+        <v>46129</v>
       </c>
       <c r="D282" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="E282" s="6" t="s">
+        <v>1529</v>
+      </c>
       <c r="F282" s="6" t="s">
-        <v>1534</v>
+        <v>1528</v>
       </c>
       <c r="G282" s="6"/>
       <c r="H282" s="6">
-        <v>2300000</v>
+        <v>174000</v>
       </c>
       <c r="I282" s="6" t="s">
-        <v>1530</v>
+        <v>1524</v>
       </c>
       <c r="J282" s="6" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="K282" s="3" t="s">
-        <v>1531</v>
+        <v>1525</v>
       </c>
       <c r="L282" s="3" t="s">
-        <v>1532</v>
+        <v>1526</v>
       </c>
       <c r="M282" s="3" t="s">
-        <v>1533</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="283" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -28791,38 +28843,35 @@
         <v>282</v>
       </c>
       <c r="B283" s="6">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C283" s="2">
-        <v>46131</v>
+        <v>46130</v>
       </c>
       <c r="D283" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E283" s="6" t="s">
-        <v>1538</v>
-      </c>
-      <c r="F283" s="5" t="s">
-        <v>1543</v>
+      <c r="F283" s="6" t="s">
+        <v>1534</v>
       </c>
       <c r="G283" s="6"/>
       <c r="H283" s="6">
-        <v>445000</v>
+        <v>2400000</v>
       </c>
       <c r="I283" s="6" t="s">
-        <v>1539</v>
+        <v>1530</v>
       </c>
       <c r="J283" s="6" t="s">
-        <v>1551</v>
+        <v>1537</v>
       </c>
       <c r="K283" s="3" t="s">
-        <v>1540</v>
+        <v>1531</v>
       </c>
       <c r="L283" s="3" t="s">
-        <v>1541</v>
+        <v>1532</v>
       </c>
       <c r="M283" s="3" t="s">
-        <v>1542</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="284" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -28830,40 +28879,38 @@
         <v>283</v>
       </c>
       <c r="B284" s="6">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C284" s="2">
         <v>46131</v>
       </c>
-      <c r="D284" s="6" t="s">
+      <c r="D284" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E284" s="6" t="s">
-        <v>1550</v>
-      </c>
-      <c r="F284" s="6" t="s">
-        <v>1548</v>
-      </c>
-      <c r="G284" s="6" t="s">
-        <v>1549</v>
-      </c>
+        <v>1538</v>
+      </c>
+      <c r="F284" s="5" t="s">
+        <v>1543</v>
+      </c>
+      <c r="G284" s="6"/>
       <c r="H284" s="6">
-        <v>441000</v>
+        <v>593000</v>
       </c>
       <c r="I284" s="6" t="s">
-        <v>1544</v>
+        <v>1539</v>
       </c>
       <c r="J284" s="6" t="s">
-        <v>1552</v>
+        <v>1551</v>
       </c>
       <c r="K284" s="3" t="s">
-        <v>1545</v>
+        <v>1540</v>
       </c>
       <c r="L284" s="3" t="s">
-        <v>1546</v>
+        <v>1541</v>
       </c>
       <c r="M284" s="3" t="s">
-        <v>1547</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="285" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
@@ -28871,7 +28918,7 @@
         <v>284</v>
       </c>
       <c r="B285" s="6">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C285" s="2">
         <v>46131</v>
@@ -28880,28 +28927,66 @@
         <v>39</v>
       </c>
       <c r="E285" s="6" t="s">
+        <v>1550</v>
+      </c>
+      <c r="F285" s="6" t="s">
+        <v>1548</v>
+      </c>
+      <c r="G285" s="6" t="s">
+        <v>1549</v>
+      </c>
+      <c r="H285" s="6">
+        <v>530000</v>
+      </c>
+      <c r="I285" s="6" t="s">
+        <v>1544</v>
+      </c>
+      <c r="J285" s="6" t="s">
+        <v>1552</v>
+      </c>
+      <c r="K285" s="3" t="s">
+        <v>1545</v>
+      </c>
+      <c r="L285" s="3" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M285" s="3" t="s">
+        <v>1547</v>
+      </c>
+    </row>
+    <row r="286" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B286" s="6">
+        <v>508</v>
+      </c>
+      <c r="C286" s="2">
+        <v>46131</v>
+      </c>
+      <c r="D286" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E286" s="6" t="s">
         <v>1554</v>
       </c>
-      <c r="F285" s="6" t="s">
+      <c r="F286" s="6" t="s">
         <v>1555</v>
       </c>
-      <c r="G285" s="6"/>
-      <c r="H285" s="6">
-        <v>245000</v>
-      </c>
-      <c r="I285" s="6" t="s">
+      <c r="G286" s="6"/>
+      <c r="H286" s="6">
+        <v>307000</v>
+      </c>
+      <c r="I286" s="6" t="s">
         <v>1553</v>
       </c>
-      <c r="J285" s="6" t="s">
+      <c r="J286" s="6" t="s">
         <v>1559</v>
       </c>
-      <c r="K285" s="3" t="s">
+      <c r="K286" s="3" t="s">
         <v>1556</v>
       </c>
-      <c r="L285" s="3" t="s">
+      <c r="L286" s="3" t="s">
         <v>1557</v>
       </c>
-      <c r="M285" s="3" t="s">
+      <c r="M286" s="3" t="s">
         <v>1558</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize fonts, make artilugios/botin public, and update store items
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A2FFB4-913E-4F6E-92AB-F484577A4D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA243E3-1F8B-4517-BB67-8C523CADF64F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="1566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="1573">
   <si>
     <t>id</t>
   </si>
@@ -18978,6 +18978,89 @@
   </si>
   <si>
     <t>https://i.postimg.cc/kgVpv5G5/501.png</t>
+  </si>
+  <si>
+    <t>rayo vallecano, laliga</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Aficionado</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rayo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: "No, a mí no, que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>yo no juego</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXgY2Jok8ja/</t>
+  </si>
+  <si>
+    <t>¡Momento digno de La Sotanita!</t>
+  </si>
+  <si>
+    <t>En el partido de liga entre el Rayo Vallecano y el Espanyol disputado en el Estadio de Vallecas, el centrocampista Óscar Valentín realizó este desacertado pase que parecía más dirigido hacia la grada que hacia un compañero, lo que provocó que un aficionado le hiciera gestos haciéndole saber que él no jugaba.</t>
+  </si>
+  <si>
+    <t>El encuentro terminó en 1-0 a favor del Rayo Vallecano con gol de Sergio Camello en el minuto 87.</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/tRr3dNG1/516.png</t>
   </si>
 </sst>
 </file>
@@ -19392,7 +19475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S286"/>
+  <dimension ref="A1:S287"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -25702,7 +25785,7 @@
       </c>
       <c r="G196" s="1"/>
       <c r="H196" s="1">
-        <v>90000</v>
+        <v>91000</v>
       </c>
       <c r="I196" s="1" t="s">
         <v>978</v>
@@ -25966,7 +26049,7 @@
       </c>
       <c r="G204" s="1"/>
       <c r="H204" s="1">
-        <v>470000</v>
+        <v>471000</v>
       </c>
       <c r="I204" s="1" t="s">
         <v>1021</v>
@@ -26409,7 +26492,7 @@
       </c>
       <c r="G217" s="1"/>
       <c r="H217" s="1">
-        <v>245000</v>
+        <v>246000</v>
       </c>
       <c r="I217" s="1" t="s">
         <v>1094</v>
@@ -26507,7 +26590,7 @@
       </c>
       <c r="G220" s="1"/>
       <c r="H220" s="1">
-        <v>427000</v>
+        <v>428000</v>
       </c>
       <c r="I220" s="1" t="s">
         <v>1111</v>
@@ -26781,7 +26864,7 @@
       </c>
       <c r="G228" s="1"/>
       <c r="H228" s="1">
-        <v>150000</v>
+        <v>151000</v>
       </c>
       <c r="I228" s="1" t="s">
         <v>1157</v>
@@ -27529,7 +27612,7 @@
       </c>
       <c r="G248" s="1"/>
       <c r="H248" s="1">
-        <v>783000</v>
+        <v>784000</v>
       </c>
       <c r="I248" s="1" t="s">
         <v>1289</v>
@@ -27816,7 +27899,7 @@
         <v>1336</v>
       </c>
       <c r="H256" s="1">
-        <v>743000</v>
+        <v>744000</v>
       </c>
       <c r="I256" s="1" t="s">
         <v>1337</v>
@@ -27891,7 +27974,7 @@
       </c>
       <c r="G258" s="1"/>
       <c r="H258" s="1">
-        <v>130000</v>
+        <v>131000</v>
       </c>
       <c r="I258" s="1" t="s">
         <v>1350</v>
@@ -28076,7 +28159,7 @@
       </c>
       <c r="G263" s="1"/>
       <c r="H263" s="1">
-        <v>287000</v>
+        <v>288000</v>
       </c>
       <c r="I263" s="1" t="s">
         <v>1383</v>
@@ -28229,7 +28312,7 @@
       </c>
       <c r="G267" s="1"/>
       <c r="H267" s="1">
-        <v>130000</v>
+        <v>131000</v>
       </c>
       <c r="I267" s="1" t="s">
         <v>1409</v>
@@ -28426,7 +28509,7 @@
       </c>
       <c r="G272" s="1"/>
       <c r="H272" s="1">
-        <v>733000</v>
+        <v>734000</v>
       </c>
       <c r="I272" s="1" t="s">
         <v>1446</v>
@@ -28506,7 +28589,7 @@
       </c>
       <c r="G274" s="1"/>
       <c r="H274" s="1">
-        <v>205000</v>
+        <v>206000</v>
       </c>
       <c r="I274" s="1" t="s">
         <v>1461</v>
@@ -28547,7 +28630,7 @@
         <v>1468</v>
       </c>
       <c r="H275" s="1">
-        <v>789000</v>
+        <v>790000</v>
       </c>
       <c r="I275" s="1" t="s">
         <v>1469</v>
@@ -28589,7 +28672,7 @@
       </c>
       <c r="G276" s="1"/>
       <c r="H276" s="1">
-        <v>1200000</v>
+        <v>1300000</v>
       </c>
       <c r="I276" s="1" t="s">
         <v>1477</v>
@@ -28628,7 +28711,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>7000000</v>
+        <v>7300000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28667,7 +28750,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>917000</v>
+        <v>950000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28706,7 +28789,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>997000</v>
+        <v>998000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28745,7 +28828,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>87000</v>
+        <v>92000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1562</v>
@@ -28781,7 +28864,7 @@
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>188000</v>
+        <v>200000</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>1518</v>
@@ -28820,7 +28903,7 @@
       </c>
       <c r="G282" s="6"/>
       <c r="H282" s="6">
-        <v>174000</v>
+        <v>177000</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>1524</v>
@@ -28895,7 +28978,7 @@
       </c>
       <c r="G284" s="6"/>
       <c r="H284" s="6">
-        <v>593000</v>
+        <v>601000</v>
       </c>
       <c r="I284" s="6" t="s">
         <v>1539</v>
@@ -28936,7 +29019,7 @@
         <v>1549</v>
       </c>
       <c r="H285" s="6">
-        <v>530000</v>
+        <v>537000</v>
       </c>
       <c r="I285" s="6" t="s">
         <v>1544</v>
@@ -28955,6 +29038,9 @@
       </c>
     </row>
     <row r="286" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A286">
+        <v>285</v>
+      </c>
       <c r="B286" s="6">
         <v>508</v>
       </c>
@@ -28972,7 +29058,7 @@
       </c>
       <c r="G286" s="6"/>
       <c r="H286" s="6">
-        <v>307000</v>
+        <v>308000</v>
       </c>
       <c r="I286" s="6" t="s">
         <v>1553</v>
@@ -28988,6 +29074,45 @@
       </c>
       <c r="M286" s="3" t="s">
         <v>1558</v>
+      </c>
+    </row>
+    <row r="287" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A287">
+        <v>286</v>
+      </c>
+      <c r="B287" s="6">
+        <v>516</v>
+      </c>
+      <c r="C287" s="2">
+        <v>46136</v>
+      </c>
+      <c r="D287" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E287" s="6" t="s">
+        <v>1566</v>
+      </c>
+      <c r="F287" s="6" t="s">
+        <v>1567</v>
+      </c>
+      <c r="G287" s="6"/>
+      <c r="H287" s="6">
+        <v>114000</v>
+      </c>
+      <c r="I287" s="6" t="s">
+        <v>1568</v>
+      </c>
+      <c r="J287" s="6" t="s">
+        <v>1572</v>
+      </c>
+      <c r="K287" s="3" t="s">
+        <v>1569</v>
+      </c>
+      <c r="L287" s="3" t="s">
+        <v>1570</v>
+      </c>
+      <c r="M287" s="3" t="s">
+        <v>1571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update news database and add components
</commit_message>
<xml_diff>
--- a/BBDD NEWS.xlsx
+++ b/BBDD NEWS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA243E3-1F8B-4517-BB67-8C523CADF64F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B20173-410B-45F9-A932-B9D2B47D2A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1814" uniqueCount="1573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1953" uniqueCount="1693">
   <si>
     <t>id</t>
   </si>
@@ -19061,6 +19061,1253 @@
   </si>
   <si>
     <t>https://i.postimg.cc/tRr3dNG1/516.png</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXeq7UBkzhH/</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pues menos mal que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>no</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> le </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gustaba hablar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mucho…</t>
+    </r>
+  </si>
+  <si>
+    <t>Take Kubo es único</t>
+  </si>
+  <si>
+    <t>Hay que proteger a Take Kubo a toda costa...</t>
+  </si>
+  <si>
+    <t>La Real Sociedad alzó la Copa del Rey este fin de semana y su plantilla lo celebró por todo lo grande.</t>
+  </si>
+  <si>
+    <t>Uno de los que más momentos históricos nos está dando cada vez que agarra el micrófono es el japonés Take Kubo, y estas fueron sus palabras para la afición.</t>
+  </si>
+  <si>
+    <t>copa del rey, real sociedad, take kubo</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXjYfHhkxGb/</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cómo olvidar cuando </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ballesteros</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> le ganó un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sprint</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cristiano</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> prime</t>
+    </r>
+  </si>
+  <si>
+    <t>Corría el año 2011 cuando un pletórico Cristiano Ronaldo de 26 años en su prime físico, cursando su cuarta temporada en el Real Madrid, se enfrentó contra un Sergio Ballesteros de 36 años con los huevos negros, y no tuvo nada que hacer ante su velocidad punta.</t>
+  </si>
+  <si>
+    <t>Se trataba de un Levante - Real Madrid en la jornada 4 de LaLiga. En la mítica temporada madridista en la que lograron 100 puntos, tuvieron este tropiezo a principios de temporada perdiendo contra el Levante 1-0.</t>
+  </si>
+  <si>
+    <t>Cristiano había entrado en la segunda parte para intentar conseguir la victoria, mientras que Ballesteros llevaba desde el inicio del partido. En el minuto 68 llegó el gol del Levante, y tan solo 10 minutos más tarde Ballesteros nos dejó claro que la victoria iba a ser para el Levante, y defendió ese resultado con energías sacadas de a saber dónde, ganándole un sprint al mismísimo Cristiano Ronaldo pese a la diferencia de edad y a la diferencia de cansancio en ese partido. Un momento icónico de LaLiga.</t>
+  </si>
+  <si>
+    <t>laliga, real madrid, getafe, sergio ballesteros, cristiano ronaldo</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXjmCQgExLq/</t>
+  </si>
+  <si>
+    <t>Tras el empate entre el Betis y el Real Madrid, el futbolista Camavinga y el presidente de su equipo Florentino Pérez, salieron a disfrutar un poco de la Feria de Abril celebrada en Sevilla.</t>
+  </si>
+  <si>
+    <t>Se pudo ver al centrocampista "blanco" demostrando que goza de talento bailando (a diferencia de jugando a fútbol), y perreando hasta abajo una canción de Bad Gyal en la Feria de Abril.</t>
+  </si>
+  <si>
+    <t>Se rumorea que tras esta noche de pasión entre ambos, se podría venir una renovación con un generoso aumento de sueldo en el contrato del francés.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camavinga</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Florentino</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dándolo todo en la </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Feria de Sevilla</t>
+    </r>
+  </si>
+  <si>
+    <t>real madrid, camavinga, florentino, feria de abril</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXj1tljE-rJ/</t>
+  </si>
+  <si>
+    <t>El que lleva apenas un mes siendo entrenador del Sevilla F.C. ha salido a dar estas sonadas declaraciones en las que se compara con los autistas.</t>
+  </si>
+  <si>
+    <t>Compara su hiperfijación y su obsesión con el trabajo con pertenecer al espectro autista, tras lo que rápidamente pide disculpas y tira la mítica carta de "tengo un familiar que lo es".</t>
+  </si>
+  <si>
+    <t>Puede que la verdadera hiperfijación del entrenador sea con la liga Hypermotion, ya que a día de hoy el Sevilla FC se encuentra en posición de descenso y puede que no siga en primera división el año que viene.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Entrenador</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sevilla</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: "Parezco un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>autista</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>sevilla, autismo, laliga</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/bwnrG2tB/512.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/8zvcFr6n/519.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/2SWyqBZJ/520.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/kgSGVtbH/521.png</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXhLAtEk0S-/</t>
+  </si>
+  <si>
+    <t>Esta es una de esas estadísticas curiosas del fútbol.</t>
+  </si>
+  <si>
+    <t>El palmarés combinado de los dos franceses Kylian Mbappé, que actualmente milita en el Real Madrid, y Ousmane Dembélé que actualmente milita en el PSG, incluye, entre otras cosas, lo siguiente:</t>
+  </si>
+  <si>
+    <t>1 Balón de Oro que recibió Dembélé este último año.</t>
+  </si>
+  <si>
+    <t>1 título de la Champions que alzó Dembélé la temporada pasada con el PSG.</t>
+  </si>
+  <si>
+    <t>3 títulos de LaLiga que ganó Dembélé en su paso por el FC Barcelona.</t>
+  </si>
+  <si>
+    <t>Mbappé, con sus 7 temporadas en el PSG y sus 2 temporadas en el Real Madrid, todavía no ha logrado coleccionar ninguno de esos tres galardones. Para pensar.</t>
+  </si>
+  <si>
+    <t>Y nada lo tiene Mbappé</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Balón de oro</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, 1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Champions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y 3 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>títulos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LaLiga</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en una sola foto</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXlsC1lk_nr/</t>
+  </si>
+  <si>
+    <t>Esto ha ocurrido durante el Talavera - Real Madrid Castilla de Primera RFEF.</t>
+  </si>
+  <si>
+    <t>El delantero de 21 años Pol Fortuny marcó un doblete para darle la victoria al Real Madrid Castilla, y durante la celebración del segundo gol con sus compañeros en la banda del campo, la primera línea de aficionados lo celebró tanto que se vino literalmente abajo la valla, y tras ella, los aficionados.</t>
+  </si>
+  <si>
+    <t>A los jugadores del Castilla se la turbopelaba el hecho y prosiguieron con su vaina.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>valla</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> se viene literalmente </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>abajo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y a los jugadores se la </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>turbopela</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXl7pKfk_6P/</t>
+  </si>
+  <si>
+    <t>Esto ha ocurrido en la Final de la Champions asiática.</t>
+  </si>
+  <si>
+    <t>El Al-Ahli de Arabia Saudí se enfrentó al Machida Zelvia de Japón, en la final de un torneo que acabó coronando el equipo árabe gracias a un gol de Firas Al-Buraikan en la prórroga.</t>
+  </si>
+  <si>
+    <t>Se pudo vivir este estrambótico momento en el que tres jugadores del Machida llevaron a cabo esta jugada ensayada con bastantes complicaciones, hasta tal punto que parecía más que estaban jugando a los bolos que al fútbol. Dos de ellos chocaron frontalmente y cayeron desplomados al suelo, a lo que acto seguido el tercero en discordia se tiró también al suelo para no dejarlos solos.</t>
+  </si>
+  <si>
+    <t>Estamos ante una jugada ensayada que no te firma ni Pep Guardiola con el mejor Manchester City ni Luis Enrique con el mejor PSG.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>jugada ensayada</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> parecía más de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>bolos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> que de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>fútbol</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXm8A6dE7xj/</t>
+  </si>
+  <si>
+    <t>Así es la liga Hypertensiones.</t>
+  </si>
+  <si>
+    <t>El S.D. Huesca - Real Zaragoza de LaLiga Hypermotion de hoy ha estado especialmente calentito.</t>
+  </si>
+  <si>
+    <t>Ambos equipos se juegan el descenso y este partido a finales de temporada es decisivo.</t>
+  </si>
+  <si>
+    <t>Tanto es así, que ha habido un momento con el partido prácticamente acabado en el que hasta el portero del Real Zaragoza, Esteban Andrada, ante la derrota 1-0 por el gol de penalti de Oscar Sielva en el minuto 65, se ha visto sobrepasado, se ha calentado que flipas y ha empujado al defensa y capitán del Huesca, Jorge Pulido, tirándolo al suelo. El colegiado le ha hecho saber que lo expulsaba con una tarjeta roja, y Andrada ha dicho "pues que me quiten lo bailado" y ha aprovechado para acabar la faena derribando del todo a Pulido, tras lo que se ha formado una trifulca interesante.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">"Ya que me </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>expulsan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, que me quiten lo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>bailao</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXnEJLGkye0/</t>
+  </si>
+  <si>
+    <t>Esteban Andrada, el portero del Real Zaragoza, le ha propinado un contundente derechazo a Jorge Pulido del S.D. Huesca tras una roja que vio desproporcionada tras empujar al césped a dicho jugador rival.</t>
+  </si>
+  <si>
+    <t>Pensó "Ya que me expulsan, que lo hagan con razones de sobra" y se lanzó a acabar el trabajo cargando el puño en contra del contrincante con el que había tenido el roce.</t>
+  </si>
+  <si>
+    <t>Se trata de dos equipos peleando el descenso en LaLiga Hypermotion, y la locura colectiva de los aficionados del Real Zaragoza no ha impedido que vivan el momento en el bar del vídeo como si se tratase de La Velada de Ibai y fuese Illojuan quien le da el puñetazo a TheGrefg.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Así se ha vivido el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>derechazo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> del portero del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Real Zaragoza</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXoU8NXjHu6/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXouE2_DM8I/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXq3ARFEzyO/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DXuO3VWk0fS/</t>
+  </si>
+  <si>
+    <r>
+      <t>Golazo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> del </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Arsenal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> femenino en la </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Champions</t>
+    </r>
+  </si>
+  <si>
+    <t>Imposible de parar</t>
+  </si>
+  <si>
+    <t>En la Champions femenina se acaba de dar uno de esos goles imposiles de parar.</t>
+  </si>
+  <si>
+    <t>Le tocaba al Arsenal chutar un tiro libre en el minuto 57 y lo colocó en un ángulo imposible de parar.</t>
+  </si>
+  <si>
+    <t>Para nada fue culpa de la habilidad de la portera, quien sin duda lo dio todo.</t>
+  </si>
+  <si>
+    <t>femenino, arsenal, champions</t>
+  </si>
+  <si>
+    <t>El portero del Real Zaragoza, Esteban Andrada, protagonizó ayer una acción bastante criminal en la que noqueó con un certero puñetazo a un jugador del S.D. Huesca peleando el descenso de la segunda división española.</t>
+  </si>
+  <si>
+    <t>Pues al parecer, el futbolista acarrea un historial bastante curioso. No contento con haber jugado en el Monterrey de la liga mexicana, resulta que también ha sido violento anteriormente en LaLiga Hypermotion, como se puede apreciar en el vídeo.</t>
+  </si>
+  <si>
+    <t>Para sus compañeros de equipo, la calentada de ayer con Jorge Pulido debe ser simplemente la cereza sobre el pastel, the cherry on the top como dicen los jóvenes de ahora.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Andrada</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ya tenía </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>antecedentes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> penales</t>
+    </r>
+  </si>
+  <si>
+    <t>hypermotion, real zaragoza, andrada</t>
+  </si>
+  <si>
+    <t>El aura que maneja Chiqui Ibai es de otro mundo.</t>
+  </si>
+  <si>
+    <t>El Galatasaray jugó recientemente un partido contra el Fenerbahçe que terminó con una paliza 3-0 en la que marcaron Victor Oshimen (el gemelo de Kolderiu), Yilmaz y Lucas Torreira.</t>
+  </si>
+  <si>
+    <t>En el inicio del partido, los jugadores realizaron el clásico paseo con niños del equipo rival agarrados de la mano, y los jugadores del Galatasaray tuvieron que soportar a un inesperado pequeñajo que les vaciló en la cara.</t>
+  </si>
+  <si>
+    <t>Se trataba de nada más y nada menos que el travieso de Chiqui Ibai, el cual se encuentra actualmente en un cambio físico interminable, para lo que ha ido a Turquía a implantarse pelo y hacer looksmaxxing, con lo que ha podido aprovechar y asistir a un partido de la liga turca.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">El </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Chiqui Ibai turco</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> manda a callar a los rivales</t>
+    </r>
+  </si>
+  <si>
+    <t>chiqui ibai, galatasaray</t>
+  </si>
+  <si>
+    <t>Enzo Fernández se acercó a saludar a la familia de Jude Bellingham en el Mutua Madrid Open.</t>
+  </si>
+  <si>
+    <t>Muchos aficionados se percataron de que el argentino saludó tanto a Jude como a Jobe (los Zipi y Zape británicos) pero no saludó a Vinicius Jr. que se encontraba ahí también, pero es que no se trataba de Vini, se trataba de la madre de los Bellingham.</t>
+  </si>
+  <si>
+    <t>Denise Bellingham iba caracterizada así porque se está preparando para un papel en la gran pantalla. Se enfrentará al reto actoral de interpretar al astro brasileño del Real Madrid, a Mr. Champions, en su biopic que llegará a todos los cines el 30 de febrero del próximo año.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">madre </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bellingham</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hará de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Vinicius</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en su nuevo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>biopic</t>
+    </r>
+  </si>
+  <si>
+    <t>bellingham, real madrid, vinicius, tenis</t>
+  </si>
+  <si>
+    <t>real madrid</t>
+  </si>
+  <si>
+    <t>bolos, japón</t>
+  </si>
+  <si>
+    <t>dembélé, mbappé</t>
+  </si>
+  <si>
+    <t>malasia</t>
+  </si>
+  <si>
+    <t>kanye west</t>
+  </si>
+  <si>
+    <t>israel, bosnia</t>
+  </si>
+  <si>
+    <t>mundial, gyökeres, suecia</t>
+  </si>
+  <si>
+    <t>ishowspeed</t>
+  </si>
+  <si>
+    <t>kanye west, bad bunny, tainy, reggaeton</t>
+  </si>
+  <si>
+    <t>trump, netanyahu, roblox, israel, usa</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DX1Rw6vz4Kq/</t>
+  </si>
+  <si>
+    <t>Un aficionado se topó con el mítico futbolista argentino Gonzalo 'Pipita' Higuaín en el Decathlon de Majadahonda.</t>
+  </si>
+  <si>
+    <t>El exfutbolista que pasó por equipos como el Real Madrid, Napoli, Juventus, AC Milan o Chelsea, se encuentra actualmente con 38 años y viviendo una vida alejada de los focos.</t>
+  </si>
+  <si>
+    <t>Es curioso ver a alguien que ha sido de talla mundial con un estado físico dejado, desaliñado, calvo como una sepia y con estas pintas. Hace apenas tres años estaba acabando su carrera profesional en el Inter Miami, antes de que llegara Leo Messi.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Este es el estado </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>físico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> actual del pipita </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Higuaín</t>
+    </r>
+  </si>
+  <si>
+    <t>higuaín, argentina, real madrid</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DX4Xt_lzBvz/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DX65C0OTJO7/</t>
+  </si>
+  <si>
+    <t>El delantero Thomasz Skublak del Inter Toronto marcó un golazo ante el Atlético Ottawa en la Premier League Canadiense.</t>
+  </si>
+  <si>
+    <t>Cuando se acercó a la banda para celebrar, optó por sacarse del calcetín su tarjeta de visita de su segundo trabajo: agente inmobiliario.</t>
+  </si>
+  <si>
+    <t>El futbolista aprovechó el momento para publicitar su otro trabajo, y salió mucho mejor de lo esperado, ya que el vídeo está dando la vuelta al mundo.</t>
+  </si>
+  <si>
+    <t>Esta es una de esas jugadas que demuestran el alto IQ futbolístico con el que cuenta Robert Lewandowski.</t>
+  </si>
+  <si>
+    <t>Al delantero polaco está en la tercera edad y ha decidido volcar todo su IQ para encontrar la forma de no tener que correr.</t>
+  </si>
+  <si>
+    <t>En esta jugada se aprecia cómo le indica a Fermín que haga un sprint al área para que los defensas se tiren sobre él y así se queda con el espacio libre para recibir el pase de Raphinha y chutar. High IQ play.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lewandowski</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> le dice a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fermín</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> que corra para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>confundir</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a los rivales</t>
+    </r>
+  </si>
+  <si>
+    <t>lewandowski, fermín, barça, laliga</t>
+  </si>
+  <si>
+    <t>canadá</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Marca </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gol</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y aprovecha para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>publicitarse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> como </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>agente inmobiliario</t>
+    </r>
+  </si>
+  <si>
+    <t>ábalos</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reel/DX6sDSNgnac/</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Vivimos en un </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pais</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en el que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>amar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>delito</t>
+    </r>
+  </si>
+  <si>
+    <t>José Luis Ábalos sigue bajo el escrutinio público cuando su único delito ha sido amar demasiado.</t>
+  </si>
+  <si>
+    <t>El que fue secretario de organización del Partido Socialista Obrero Español y mano derecha de Pedro Sánchez se encuentra hoy en día encarcelado junto a Nicolás Maduro y Diddy en la prisión de Soto del Real.</t>
+  </si>
+  <si>
+    <t>El caso Ábalos sigue juicio tras juicio y se está persiguiendo a un hombre familiar, romántico, y ante todo patriota. FREE ÁBALOS.</t>
   </si>
 </sst>
 </file>
@@ -19475,7 +20722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S287"/>
+  <dimension ref="A1:S304"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" customWidth="1"/>
@@ -20433,7 +21680,7 @@
         <v>148</v>
       </c>
       <c r="H31" s="1">
-        <v>533000</v>
+        <v>534000</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>149</v>
@@ -22393,7 +23640,7 @@
       </c>
       <c r="G96" s="1"/>
       <c r="H96" s="1">
-        <v>766000</v>
+        <v>767000</v>
       </c>
       <c r="I96" s="1" t="s">
         <v>425</v>
@@ -22455,7 +23702,7 @@
       </c>
       <c r="G98" s="1"/>
       <c r="H98" s="1">
-        <v>204000</v>
+        <v>205000</v>
       </c>
       <c r="I98" s="1" t="s">
         <v>434</v>
@@ -22968,7 +24215,7 @@
       </c>
       <c r="G113" s="1"/>
       <c r="H113" s="1">
-        <v>544000</v>
+        <v>545000</v>
       </c>
       <c r="I113" s="1" t="s">
         <v>516</v>
@@ -23135,7 +24382,7 @@
       </c>
       <c r="G118" s="1"/>
       <c r="H118" s="1">
-        <v>441000</v>
+        <v>442000</v>
       </c>
       <c r="I118" s="1" t="s">
         <v>543</v>
@@ -23465,7 +24712,7 @@
         <v>599</v>
       </c>
       <c r="H127" s="1">
-        <v>996000</v>
+        <v>997000</v>
       </c>
       <c r="I127" s="1" t="s">
         <v>600</v>
@@ -23745,7 +24992,7 @@
       </c>
       <c r="G135" s="1"/>
       <c r="H135" s="1">
-        <v>421000</v>
+        <v>422000</v>
       </c>
       <c r="I135" s="1" t="s">
         <v>646</v>
@@ -24217,7 +25464,7 @@
       </c>
       <c r="G149" s="1"/>
       <c r="H149" s="1">
-        <v>238000</v>
+        <v>239000</v>
       </c>
       <c r="I149" s="1" t="s">
         <v>722</v>
@@ -24384,7 +25631,7 @@
         <v>748</v>
       </c>
       <c r="H154" s="1">
-        <v>108000</v>
+        <v>110000</v>
       </c>
       <c r="I154" s="1" t="s">
         <v>749</v>
@@ -24846,7 +26093,7 @@
       </c>
       <c r="G167" s="1"/>
       <c r="H167" s="1">
-        <v>171000</v>
+        <v>172000</v>
       </c>
       <c r="I167" s="1" t="s">
         <v>828</v>
@@ -25042,7 +26289,7 @@
       </c>
       <c r="G173" s="1"/>
       <c r="H173" s="1">
-        <v>728000</v>
+        <v>729000</v>
       </c>
       <c r="I173" s="1" t="s">
         <v>862</v>
@@ -25327,7 +26574,7 @@
       </c>
       <c r="G182" s="1"/>
       <c r="H182" s="1">
-        <v>93000</v>
+        <v>94000</v>
       </c>
       <c r="I182" s="1" t="s">
         <v>906</v>
@@ -25429,7 +26676,7 @@
       </c>
       <c r="G185" s="1"/>
       <c r="H185" s="1">
-        <v>82000</v>
+        <v>83000</v>
       </c>
       <c r="I185" s="1" t="s">
         <v>923</v>
@@ -25950,7 +27197,7 @@
       </c>
       <c r="G201" s="1"/>
       <c r="H201" s="1">
-        <v>276000</v>
+        <v>277000</v>
       </c>
       <c r="I201" s="1" t="s">
         <v>1005</v>
@@ -25983,7 +27230,7 @@
       </c>
       <c r="G202" s="1"/>
       <c r="H202" s="1">
-        <v>584000</v>
+        <v>585000</v>
       </c>
       <c r="I202" s="1" t="s">
         <v>1010</v>
@@ -26253,7 +27500,7 @@
       </c>
       <c r="G210" s="1"/>
       <c r="H210" s="1">
-        <v>340000</v>
+        <v>342000</v>
       </c>
       <c r="I210" s="1" t="s">
         <v>1056</v>
@@ -26525,7 +27772,7 @@
       </c>
       <c r="G218" s="1"/>
       <c r="H218" s="1">
-        <v>412000</v>
+        <v>413000</v>
       </c>
       <c r="I218" s="1" t="s">
         <v>1099</v>
@@ -26689,7 +27936,7 @@
       </c>
       <c r="G223" s="1"/>
       <c r="H223" s="1">
-        <v>99000</v>
+        <v>100000</v>
       </c>
       <c r="I223" s="1" t="s">
         <v>1128</v>
@@ -26720,6 +27967,9 @@
       <c r="D224" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="E224" s="6" t="s">
+        <v>1668</v>
+      </c>
       <c r="F224" s="1" t="s">
         <v>1133</v>
       </c>
@@ -26753,12 +28003,15 @@
       <c r="D225" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="E225" s="6" t="s">
+        <v>1667</v>
+      </c>
       <c r="F225" s="1" t="s">
         <v>1138</v>
       </c>
       <c r="G225" s="1"/>
       <c r="H225" s="1">
-        <v>264000</v>
+        <v>265000</v>
       </c>
       <c r="I225" s="1" t="s">
         <v>1139</v>
@@ -26789,6 +28042,9 @@
       <c r="D226" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="E226" s="6" t="s">
+        <v>1666</v>
+      </c>
       <c r="F226" s="1" t="s">
         <v>1144</v>
       </c>
@@ -26796,7 +28052,7 @@
         <v>1145</v>
       </c>
       <c r="H226" s="1">
-        <v>89000</v>
+        <v>90000</v>
       </c>
       <c r="I226" s="1" t="s">
         <v>1146</v>
@@ -26824,6 +28080,9 @@
       <c r="D227" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="E227" s="6" t="s">
+        <v>1665</v>
+      </c>
       <c r="F227" s="1" t="s">
         <v>1150</v>
       </c>
@@ -26859,12 +28118,15 @@
       <c r="D228" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="E228" s="6" t="s">
+        <v>1664</v>
+      </c>
       <c r="F228" s="1" t="s">
         <v>1156</v>
       </c>
       <c r="G228" s="1"/>
       <c r="H228" s="1">
-        <v>151000</v>
+        <v>152000</v>
       </c>
       <c r="I228" s="1" t="s">
         <v>1157</v>
@@ -26894,6 +28156,9 @@
       </c>
       <c r="D229" s="1" t="s">
         <v>31</v>
+      </c>
+      <c r="E229" s="6" t="s">
+        <v>1663</v>
       </c>
       <c r="F229" s="1" t="s">
         <v>1162</v>
@@ -27426,7 +28691,7 @@
         <v>1256</v>
       </c>
       <c r="H243" s="1">
-        <v>387000</v>
+        <v>388000</v>
       </c>
       <c r="I243" s="1" t="s">
         <v>1257</v>
@@ -27465,7 +28730,7 @@
       </c>
       <c r="G244" s="1"/>
       <c r="H244" s="1">
-        <v>184000</v>
+        <v>185000</v>
       </c>
       <c r="I244" s="1" t="s">
         <v>1264</v>
@@ -27899,7 +29164,7 @@
         <v>1336</v>
       </c>
       <c r="H256" s="1">
-        <v>744000</v>
+        <v>746000</v>
       </c>
       <c r="I256" s="1" t="s">
         <v>1337</v>
@@ -28120,7 +29385,7 @@
       </c>
       <c r="G262" s="1"/>
       <c r="H262" s="1">
-        <v>501000</v>
+        <v>502000</v>
       </c>
       <c r="I262" s="1" t="s">
         <v>1376</v>
@@ -28159,7 +29424,7 @@
       </c>
       <c r="G263" s="1"/>
       <c r="H263" s="1">
-        <v>288000</v>
+        <v>289000</v>
       </c>
       <c r="I263" s="1" t="s">
         <v>1383</v>
@@ -28195,7 +29460,7 @@
       </c>
       <c r="G264" s="1"/>
       <c r="H264" s="1">
-        <v>135000</v>
+        <v>136000</v>
       </c>
       <c r="I264" s="1" t="s">
         <v>1389</v>
@@ -28509,7 +29774,7 @@
       </c>
       <c r="G272" s="1"/>
       <c r="H272" s="1">
-        <v>734000</v>
+        <v>741000</v>
       </c>
       <c r="I272" s="1" t="s">
         <v>1446</v>
@@ -28589,7 +29854,7 @@
       </c>
       <c r="G274" s="1"/>
       <c r="H274" s="1">
-        <v>206000</v>
+        <v>272000</v>
       </c>
       <c r="I274" s="1" t="s">
         <v>1461</v>
@@ -28711,7 +29976,7 @@
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="1">
-        <v>7300000</v>
+        <v>8200000</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>1484</v>
@@ -28750,7 +30015,7 @@
       </c>
       <c r="G278" s="6"/>
       <c r="H278" s="1">
-        <v>950000</v>
+        <v>1000000</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>1509</v>
@@ -28789,7 +30054,7 @@
       </c>
       <c r="G279" s="6"/>
       <c r="H279" s="6">
-        <v>998000</v>
+        <v>1000000</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>1502</v>
@@ -28828,7 +30093,7 @@
       </c>
       <c r="G280" s="6"/>
       <c r="H280" s="6">
-        <v>92000</v>
+        <v>102000</v>
       </c>
       <c r="I280" s="6" t="s">
         <v>1562</v>
@@ -28864,7 +30129,7 @@
       </c>
       <c r="G281" s="6"/>
       <c r="H281" s="6">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>1518</v>
@@ -28903,7 +30168,7 @@
       </c>
       <c r="G282" s="6"/>
       <c r="H282" s="6">
-        <v>177000</v>
+        <v>188000</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>1524</v>
@@ -28934,6 +30199,9 @@
       <c r="D283" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="E283" s="6" t="s">
+        <v>1662</v>
+      </c>
       <c r="F283" s="6" t="s">
         <v>1534</v>
       </c>
@@ -28978,7 +30246,7 @@
       </c>
       <c r="G284" s="6"/>
       <c r="H284" s="6">
-        <v>601000</v>
+        <v>625000</v>
       </c>
       <c r="I284" s="6" t="s">
         <v>1539</v>
@@ -29019,7 +30287,7 @@
         <v>1549</v>
       </c>
       <c r="H285" s="6">
-        <v>537000</v>
+        <v>546000</v>
       </c>
       <c r="I285" s="6" t="s">
         <v>1544</v>
@@ -29058,7 +30326,7 @@
       </c>
       <c r="G286" s="6"/>
       <c r="H286" s="6">
-        <v>308000</v>
+        <v>312000</v>
       </c>
       <c r="I286" s="6" t="s">
         <v>1553</v>
@@ -29081,38 +30349,686 @@
         <v>286</v>
       </c>
       <c r="B287" s="6">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="C287" s="2">
-        <v>46136</v>
+        <v>46135</v>
       </c>
       <c r="D287" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E287" s="6" t="s">
+        <v>1579</v>
+      </c>
+      <c r="F287" s="6" t="s">
+        <v>1574</v>
+      </c>
+      <c r="G287" s="6" t="s">
+        <v>1575</v>
+      </c>
+      <c r="H287" s="6">
+        <v>51000</v>
+      </c>
+      <c r="I287" s="6" t="s">
+        <v>1573</v>
+      </c>
+      <c r="J287" s="6" t="s">
+        <v>1598</v>
+      </c>
+      <c r="K287" s="3" t="s">
+        <v>1576</v>
+      </c>
+      <c r="L287" s="3" t="s">
+        <v>1577</v>
+      </c>
+      <c r="M287" s="3" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="288" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A288">
+        <v>287</v>
+      </c>
+      <c r="B288" s="6">
+        <v>516</v>
+      </c>
+      <c r="C288" s="2">
+        <v>46136</v>
+      </c>
+      <c r="D288" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E288" s="6" t="s">
         <v>1566</v>
       </c>
-      <c r="F287" s="6" t="s">
+      <c r="F288" s="6" t="s">
         <v>1567</v>
       </c>
-      <c r="G287" s="6"/>
-      <c r="H287" s="6">
-        <v>114000</v>
-      </c>
-      <c r="I287" s="6" t="s">
+      <c r="G288" s="6"/>
+      <c r="H288" s="6">
+        <v>226000</v>
+      </c>
+      <c r="I288" s="6" t="s">
         <v>1568</v>
       </c>
-      <c r="J287" s="6" t="s">
+      <c r="J288" s="6" t="s">
         <v>1572</v>
       </c>
-      <c r="K287" s="3" t="s">
+      <c r="K288" s="3" t="s">
         <v>1569</v>
       </c>
-      <c r="L287" s="3" t="s">
+      <c r="L288" s="3" t="s">
         <v>1570</v>
       </c>
-      <c r="M287" s="3" t="s">
+      <c r="M288" s="3" t="s">
         <v>1571</v>
+      </c>
+    </row>
+    <row r="289" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A289">
+        <v>288</v>
+      </c>
+      <c r="B289" s="6">
+        <v>517</v>
+      </c>
+      <c r="C289" s="2">
+        <v>46136</v>
+      </c>
+      <c r="D289" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E289" s="6" t="s">
+        <v>1661</v>
+      </c>
+      <c r="F289" s="6" t="s">
+        <v>1610</v>
+      </c>
+      <c r="G289" s="6" t="s">
+        <v>1609</v>
+      </c>
+      <c r="H289" s="6">
+        <v>69000</v>
+      </c>
+      <c r="I289" s="6" t="s">
+        <v>1602</v>
+      </c>
+      <c r="K289" s="3" t="s">
+        <v>1603</v>
+      </c>
+      <c r="L289" s="3" t="s">
+        <v>1604</v>
+      </c>
+      <c r="M289" s="3" t="s">
+        <v>1605</v>
+      </c>
+      <c r="N289" s="3" t="s">
+        <v>1606</v>
+      </c>
+      <c r="O289" s="3" t="s">
+        <v>1607</v>
+      </c>
+      <c r="P289" s="3" t="s">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="290" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A290">
+        <v>289</v>
+      </c>
+      <c r="B290" s="6">
+        <v>519</v>
+      </c>
+      <c r="C290" s="2">
+        <v>46137</v>
+      </c>
+      <c r="D290" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E290" s="6" t="s">
+        <v>1585</v>
+      </c>
+      <c r="F290" s="6" t="s">
+        <v>1581</v>
+      </c>
+      <c r="G290" s="6"/>
+      <c r="H290" s="6">
+        <v>800000</v>
+      </c>
+      <c r="I290" s="6" t="s">
+        <v>1580</v>
+      </c>
+      <c r="J290" s="6" t="s">
+        <v>1599</v>
+      </c>
+      <c r="K290" s="3" t="s">
+        <v>1582</v>
+      </c>
+      <c r="L290" s="3" t="s">
+        <v>1583</v>
+      </c>
+      <c r="M290" s="3" t="s">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="291" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A291">
+        <v>290</v>
+      </c>
+      <c r="B291" s="6">
+        <v>520</v>
+      </c>
+      <c r="C291" s="2">
+        <v>46137</v>
+      </c>
+      <c r="D291" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E291" s="6" t="s">
+        <v>1591</v>
+      </c>
+      <c r="F291" s="6" t="s">
+        <v>1590</v>
+      </c>
+      <c r="G291" s="6"/>
+      <c r="H291" s="6">
+        <v>394000</v>
+      </c>
+      <c r="I291" s="6" t="s">
+        <v>1586</v>
+      </c>
+      <c r="J291" s="6" t="s">
+        <v>1600</v>
+      </c>
+      <c r="K291" s="3" t="s">
+        <v>1587</v>
+      </c>
+      <c r="L291" s="3" t="s">
+        <v>1588</v>
+      </c>
+      <c r="M291" s="3" t="s">
+        <v>1589</v>
+      </c>
+    </row>
+    <row r="292" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A292">
+        <v>291</v>
+      </c>
+      <c r="B292" s="6">
+        <v>521</v>
+      </c>
+      <c r="C292" s="2">
+        <v>46137</v>
+      </c>
+      <c r="D292" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E292" s="6" t="s">
+        <v>1597</v>
+      </c>
+      <c r="F292" s="6" t="s">
+        <v>1596</v>
+      </c>
+      <c r="G292" s="6"/>
+      <c r="H292" s="6">
+        <v>882000</v>
+      </c>
+      <c r="I292" s="6" t="s">
+        <v>1592</v>
+      </c>
+      <c r="J292" s="6" t="s">
+        <v>1601</v>
+      </c>
+      <c r="K292" s="3" t="s">
+        <v>1593</v>
+      </c>
+      <c r="L292" s="3" t="s">
+        <v>1594</v>
+      </c>
+      <c r="M292" s="3" t="s">
+        <v>1595</v>
+      </c>
+    </row>
+    <row r="293" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A293">
+        <v>292</v>
+      </c>
+      <c r="B293" s="6">
+        <v>523</v>
+      </c>
+      <c r="C293" s="2">
+        <v>46138</v>
+      </c>
+      <c r="D293" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E293" s="6" t="s">
+        <v>1659</v>
+      </c>
+      <c r="F293" s="6" t="s">
+        <v>1615</v>
+      </c>
+      <c r="G293" s="6"/>
+      <c r="H293" s="6">
+        <v>199000</v>
+      </c>
+      <c r="I293" s="6" t="s">
+        <v>1611</v>
+      </c>
+      <c r="K293" s="3" t="s">
+        <v>1612</v>
+      </c>
+      <c r="L293" s="3" t="s">
+        <v>1613</v>
+      </c>
+      <c r="M293" s="3" t="s">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="294" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A294">
+        <v>293</v>
+      </c>
+      <c r="B294" s="6">
+        <v>524</v>
+      </c>
+      <c r="C294" s="2">
+        <v>46138</v>
+      </c>
+      <c r="D294" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E294" s="6" t="s">
+        <v>1660</v>
+      </c>
+      <c r="F294" s="6" t="s">
+        <v>1621</v>
+      </c>
+      <c r="G294" s="6"/>
+      <c r="H294" s="6">
+        <v>1000000</v>
+      </c>
+      <c r="I294" s="6" t="s">
+        <v>1616</v>
+      </c>
+      <c r="K294" s="3" t="s">
+        <v>1617</v>
+      </c>
+      <c r="L294" s="3" t="s">
+        <v>1618</v>
+      </c>
+      <c r="M294" s="3" t="s">
+        <v>1619</v>
+      </c>
+      <c r="N294" s="3" t="s">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="295" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A295">
+        <v>294</v>
+      </c>
+      <c r="B295" s="6">
+        <v>526</v>
+      </c>
+      <c r="C295" s="2">
+        <v>46138</v>
+      </c>
+      <c r="D295" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E295" s="6" t="s">
+        <v>1647</v>
+      </c>
+      <c r="F295" s="6" t="s">
+        <v>1627</v>
+      </c>
+      <c r="G295" s="6"/>
+      <c r="H295" s="6">
+        <v>8300000</v>
+      </c>
+      <c r="I295" s="6" t="s">
+        <v>1622</v>
+      </c>
+      <c r="K295" s="3" t="s">
+        <v>1623</v>
+      </c>
+      <c r="L295" s="3" t="s">
+        <v>1624</v>
+      </c>
+      <c r="M295" s="3" t="s">
+        <v>1625</v>
+      </c>
+      <c r="N295" s="3" t="s">
+        <v>1626</v>
+      </c>
+    </row>
+    <row r="296" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A296">
+        <v>295</v>
+      </c>
+      <c r="B296" s="6">
+        <v>527</v>
+      </c>
+      <c r="C296" s="2">
+        <v>46138</v>
+      </c>
+      <c r="D296" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E296" s="6" t="s">
+        <v>1647</v>
+      </c>
+      <c r="F296" s="6" t="s">
+        <v>1632</v>
+      </c>
+      <c r="G296" s="6"/>
+      <c r="H296" s="6">
+        <v>174000</v>
+      </c>
+      <c r="I296" s="6" t="s">
+        <v>1628</v>
+      </c>
+      <c r="K296" s="3" t="s">
+        <v>1629</v>
+      </c>
+      <c r="L296" s="3" t="s">
+        <v>1630</v>
+      </c>
+      <c r="M296" s="3" t="s">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="297" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A297">
+        <v>296</v>
+      </c>
+      <c r="B297" s="6">
+        <v>528</v>
+      </c>
+      <c r="C297" s="2">
+        <v>46139</v>
+      </c>
+      <c r="D297" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E297" s="6" t="s">
+        <v>1642</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>1637</v>
+      </c>
+      <c r="G297" s="6" t="s">
+        <v>1638</v>
+      </c>
+      <c r="H297" s="6">
+        <v>404000</v>
+      </c>
+      <c r="I297" s="6" t="s">
+        <v>1633</v>
+      </c>
+      <c r="K297" s="3" t="s">
+        <v>1639</v>
+      </c>
+      <c r="L297" s="3" t="s">
+        <v>1640</v>
+      </c>
+      <c r="M297" s="3" t="s">
+        <v>1641</v>
+      </c>
+    </row>
+    <row r="298" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A298">
+        <v>297</v>
+      </c>
+      <c r="B298" s="6">
+        <v>529</v>
+      </c>
+      <c r="C298" s="2">
+        <v>46139</v>
+      </c>
+      <c r="D298" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E298" s="6" t="s">
+        <v>1647</v>
+      </c>
+      <c r="F298" s="6" t="s">
+        <v>1646</v>
+      </c>
+      <c r="G298" s="6"/>
+      <c r="H298" s="6">
+        <v>392000</v>
+      </c>
+      <c r="I298" s="6" t="s">
+        <v>1634</v>
+      </c>
+      <c r="K298" s="3" t="s">
+        <v>1643</v>
+      </c>
+      <c r="L298" s="3" t="s">
+        <v>1644</v>
+      </c>
+      <c r="M298" s="3" t="s">
+        <v>1645</v>
+      </c>
+    </row>
+    <row r="299" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A299">
+        <v>298</v>
+      </c>
+      <c r="B299" s="6">
+        <v>530</v>
+      </c>
+      <c r="C299" s="2">
+        <v>46140</v>
+      </c>
+      <c r="D299" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E299" s="6" t="s">
+        <v>1653</v>
+      </c>
+      <c r="F299" s="6" t="s">
+        <v>1652</v>
+      </c>
+      <c r="G299" s="6"/>
+      <c r="H299" s="6">
+        <v>218000</v>
+      </c>
+      <c r="I299" s="6" t="s">
+        <v>1635</v>
+      </c>
+      <c r="K299" s="3" t="s">
+        <v>1648</v>
+      </c>
+      <c r="L299" s="3" t="s">
+        <v>1649</v>
+      </c>
+      <c r="M299" s="3" t="s">
+        <v>1650</v>
+      </c>
+      <c r="N299" s="3" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A300">
+        <v>299</v>
+      </c>
+      <c r="B300" s="6">
+        <v>531</v>
+      </c>
+      <c r="C300" s="2">
+        <v>46141</v>
+      </c>
+      <c r="D300" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E300" s="6" t="s">
+        <v>1658</v>
+      </c>
+      <c r="F300" s="6" t="s">
+        <v>1657</v>
+      </c>
+      <c r="G300" s="6"/>
+      <c r="H300" s="6">
+        <v>739000</v>
+      </c>
+      <c r="I300" s="6" t="s">
+        <v>1636</v>
+      </c>
+      <c r="K300" s="3" t="s">
+        <v>1654</v>
+      </c>
+      <c r="L300" s="3" t="s">
+        <v>1655</v>
+      </c>
+      <c r="M300" s="3" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="301" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A301">
+        <v>300</v>
+      </c>
+      <c r="B301" s="6">
+        <v>535</v>
+      </c>
+      <c r="C301" s="2">
+        <v>46144</v>
+      </c>
+      <c r="D301" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E301" s="6" t="s">
+        <v>1674</v>
+      </c>
+      <c r="F301" s="6" t="s">
+        <v>1673</v>
+      </c>
+      <c r="G301" s="6"/>
+      <c r="H301" s="6">
+        <v>410000</v>
+      </c>
+      <c r="I301" s="6" t="s">
+        <v>1669</v>
+      </c>
+      <c r="K301" s="3" t="s">
+        <v>1670</v>
+      </c>
+      <c r="L301" s="3" t="s">
+        <v>1671</v>
+      </c>
+      <c r="M301" s="3" t="s">
+        <v>1672</v>
+      </c>
+    </row>
+    <row r="302" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" s="6">
+        <v>538</v>
+      </c>
+      <c r="C302" s="2">
+        <v>46145</v>
+      </c>
+      <c r="D302" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E302" s="6" t="s">
+        <v>1685</v>
+      </c>
+      <c r="F302" s="6" t="s">
+        <v>1686</v>
+      </c>
+      <c r="G302" s="6"/>
+      <c r="H302" s="6">
+        <v>293000</v>
+      </c>
+      <c r="I302" s="6" t="s">
+        <v>1675</v>
+      </c>
+      <c r="K302" s="3" t="s">
+        <v>1677</v>
+      </c>
+      <c r="L302" s="3" t="s">
+        <v>1678</v>
+      </c>
+      <c r="M302" s="3" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="303" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A303">
+        <v>302</v>
+      </c>
+      <c r="B303" s="6">
+        <v>541</v>
+      </c>
+      <c r="C303" s="2">
+        <v>46146</v>
+      </c>
+      <c r="D303" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E303" s="6" t="s">
+        <v>1687</v>
+      </c>
+      <c r="F303" s="6" t="s">
+        <v>1689</v>
+      </c>
+      <c r="G303" s="6"/>
+      <c r="H303" s="6">
+        <v>62000</v>
+      </c>
+      <c r="I303" s="6" t="s">
+        <v>1688</v>
+      </c>
+      <c r="K303" s="3" t="s">
+        <v>1690</v>
+      </c>
+      <c r="L303" s="3" t="s">
+        <v>1691</v>
+      </c>
+      <c r="M303" s="3" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="304" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A304">
+        <v>303</v>
+      </c>
+      <c r="B304" s="6">
+        <v>542</v>
+      </c>
+      <c r="C304" s="2">
+        <v>46146</v>
+      </c>
+      <c r="D304" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E304" s="6" t="s">
+        <v>1684</v>
+      </c>
+      <c r="F304" s="6" t="s">
+        <v>1683</v>
+      </c>
+      <c r="G304" s="6"/>
+      <c r="H304" s="6">
+        <v>50000</v>
+      </c>
+      <c r="I304" s="6" t="s">
+        <v>1676</v>
+      </c>
+      <c r="K304" s="3" t="s">
+        <v>1680</v>
+      </c>
+      <c r="L304" s="3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="M304" s="3" t="s">
+        <v>1682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>